<commit_message>
feat: make blog word count configurable
Add a single-call word-count option and simplify draft acceptance to the requested minimum length plus placeholder detection. Include the latest completed tracker row and generated Blog 6 draft.
</commit_message>
<xml_diff>
--- a/outputs/wordpress-blog-writer-template/wordpress-blog-content-tracker.xlsx
+++ b/outputs/wordpress-blog-writer-template/wordpress-blog-content-tracker.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="42">
   <si>
     <t>Blog ID</t>
   </si>
@@ -93,6 +93,15 @@
   </si>
   <si>
     <t>C:\Users\NolanYoung\Developer\repos\Nolan-Young-local-agent-laboratory\outputs\wordpress-blog-writer-template\drafts\blog-005.md</t>
+  </si>
+  <si>
+    <t>blog-006</t>
+  </si>
+  <si>
+    <t>All of the basics of GitHub CLI commands and what they do</t>
+  </si>
+  <si>
+    <t>C:\Users\NolanYoung\Developer\repos\Nolan-Young-local-agent-laboratory\outputs\wordpress-blog-writer-template\drafts\blog-006.md</t>
   </si>
   <si>
     <t>WordPress Blog Writer — tracker instructions</t>
@@ -737,12 +746,28 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="3"/>
+    <row r="7" ht="30" customHeight="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>27</v>
+      </c>
       <c r="C7" s="3"/>
+      <c r="D7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="F7" s="4"/>
+      <c r="G7" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="H7" s="5"/>
+      <c r="I7" s="2" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
@@ -839,56 +864,56 @@
   <sheetData>
     <row r="1" ht="27.95" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B1" s="6"/>
     </row>
     <row r="2" ht="33.95" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" ht="33.95" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" ht="33.95" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" ht="33.95" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="33.95" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" ht="33.95" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>